<commit_message>
Explicit elasticity data for mobile equipment
</commit_message>
<xml_diff>
--- a/InputData/indst/EoIEPwEEI/Elasticity of Ind Eqpt Price wrt E Eff Improvements.xlsx
+++ b/InputData/indst/EoIEPwEEI/Elasticity of Ind Eqpt Price wrt E Eff Improvements.xlsx
@@ -1,34 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\EoIEPwEEI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\indst\EoIEPwEEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138C8715-36E6-4D76-B3E3-4B17A9E8069F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3217B7-465B-4D4E-B5F5-63CD0C08DA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="763" firstSheet="4" activeTab="15" xr2:uid="{05F795DA-2DEA-4188-AD09-B14B246EEF5D}"/>
+    <workbookView xWindow="1545" yWindow="1200" windowWidth="24345" windowHeight="14850" tabRatio="763" firstSheet="7" activeTab="17" xr2:uid="{05F795DA-2DEA-4188-AD09-B14B246EEF5D}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="indst motors" sheetId="15" r:id="rId2"/>
-    <sheet name="furnaces" sheetId="8" r:id="rId3"/>
-    <sheet name="comm refrigerators" sheetId="7" r:id="rId4"/>
-    <sheet name="process chillers" sheetId="12" r:id="rId5"/>
-    <sheet name="water heaters" sheetId="6" r:id="rId6"/>
-    <sheet name="pumps" sheetId="2" r:id="rId7"/>
-    <sheet name="motors" sheetId="4" r:id="rId8"/>
-    <sheet name="comm boilers" sheetId="5" r:id="rId9"/>
-    <sheet name="indst boilers" sheetId="9" r:id="rId10"/>
-    <sheet name="indst heat pumps" sheetId="11" r:id="rId11"/>
-    <sheet name="fans-blowers" sheetId="14" r:id="rId12"/>
-    <sheet name="solid fuel boilers" sheetId="16" r:id="rId13"/>
-    <sheet name="Lighting" sheetId="17" r:id="rId14"/>
-    <sheet name="calcs" sheetId="13" r:id="rId15"/>
-    <sheet name="EoIEPwEEI" sheetId="3" r:id="rId16"/>
+    <sheet name="cpi" sheetId="19" r:id="rId2"/>
+    <sheet name="indst motors" sheetId="15" r:id="rId3"/>
+    <sheet name="furnaces" sheetId="8" r:id="rId4"/>
+    <sheet name="comm refrigerators" sheetId="7" r:id="rId5"/>
+    <sheet name="process chillers" sheetId="12" r:id="rId6"/>
+    <sheet name="water heaters" sheetId="6" r:id="rId7"/>
+    <sheet name="pumps" sheetId="2" r:id="rId8"/>
+    <sheet name="motors" sheetId="4" r:id="rId9"/>
+    <sheet name="comm boilers" sheetId="5" r:id="rId10"/>
+    <sheet name="indst boilers" sheetId="9" r:id="rId11"/>
+    <sheet name="indst heat pumps" sheetId="11" r:id="rId12"/>
+    <sheet name="fans-blowers" sheetId="14" r:id="rId13"/>
+    <sheet name="solid fuel boilers" sheetId="16" r:id="rId14"/>
+    <sheet name="Lighting" sheetId="17" r:id="rId15"/>
+    <sheet name="mobile" sheetId="18" r:id="rId16"/>
+    <sheet name="calcs" sheetId="13" r:id="rId17"/>
+    <sheet name="EoIEPwEEI" sheetId="3" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1106" uniqueCount="610">
   <si>
     <t>Source:</t>
   </si>
@@ -1672,19 +1674,291 @@
   <si>
     <t>lumens</t>
   </si>
+  <si>
+    <t>Cal Poly &amp; University of Nebraska, Lincoln</t>
+  </si>
+  <si>
+    <t>Assessing the Cost and Fuel Consumption of Off-Road Agricultural Equipment</t>
+  </si>
+  <si>
+    <t>https://digitalcommons.calpoly.edu/agb_fac/161/?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>Historical Consumer Price Index for All Urban Consumers (CPI-U): U.S. city average, all items, index</t>
+  </si>
+  <si>
+    <t>averages — Continued</t>
+  </si>
+  <si>
+    <t>[1982-84=100, unless otherwise noted]</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Semiannual averages</t>
+  </si>
+  <si>
+    <t>Annual avg.</t>
+  </si>
+  <si>
+    <t>Percent change from previous</t>
+  </si>
+  <si>
+    <t>Multiply by to get 2012 Dollars</t>
+  </si>
+  <si>
+    <t>1st half</t>
+  </si>
+  <si>
+    <t>2nd half</t>
+  </si>
+  <si>
+    <t>Dec.</t>
+  </si>
+  <si>
+    <t>1968............................................................................. .</t>
+  </si>
+  <si>
+    <t>–</t>
+  </si>
+  <si>
+    <t>1969............................................................................. .</t>
+  </si>
+  <si>
+    <t>1970............................................................................. .</t>
+  </si>
+  <si>
+    <t>1971............................................................................. .</t>
+  </si>
+  <si>
+    <t>1972............................................................................. .</t>
+  </si>
+  <si>
+    <t>1973............................................................................. .</t>
+  </si>
+  <si>
+    <t>1974............................................................................. .</t>
+  </si>
+  <si>
+    <t>1975............................................................................. .</t>
+  </si>
+  <si>
+    <t>1976............................................................................. .</t>
+  </si>
+  <si>
+    <t>1977............................................................................. .</t>
+  </si>
+  <si>
+    <t>1978............................................................................. .</t>
+  </si>
+  <si>
+    <t>1979............................................................................. .</t>
+  </si>
+  <si>
+    <t>1980............................................................................. .</t>
+  </si>
+  <si>
+    <t>1981............................................................................. .</t>
+  </si>
+  <si>
+    <t>1982............................................................................. .</t>
+  </si>
+  <si>
+    <t>1983............................................................................. .</t>
+  </si>
+  <si>
+    <t>1984............................................................................. .</t>
+  </si>
+  <si>
+    <t>1985............................................................................. .</t>
+  </si>
+  <si>
+    <t>1986............................................................................. .</t>
+  </si>
+  <si>
+    <t>1987............................................................................. .</t>
+  </si>
+  <si>
+    <t>1988............................................................................. .</t>
+  </si>
+  <si>
+    <t>1989............................................................................. .</t>
+  </si>
+  <si>
+    <t>1990............................................................................. .</t>
+  </si>
+  <si>
+    <t>1991............................................................................. .</t>
+  </si>
+  <si>
+    <t>1992............................................................................. .</t>
+  </si>
+  <si>
+    <t>1993............................................................................. .</t>
+  </si>
+  <si>
+    <t>1994............................................................................. .</t>
+  </si>
+  <si>
+    <t>1995............................................................................. .</t>
+  </si>
+  <si>
+    <t>1996............................................................................. .</t>
+  </si>
+  <si>
+    <t>1997............................................................................. .</t>
+  </si>
+  <si>
+    <t>1998............................................................................. .</t>
+  </si>
+  <si>
+    <t>1999............................................................................. .</t>
+  </si>
+  <si>
+    <t>2000............................................................................. .</t>
+  </si>
+  <si>
+    <t>2001............................................................................. .</t>
+  </si>
+  <si>
+    <t>2002............................................................................. .</t>
+  </si>
+  <si>
+    <t>2003............................................................................. .</t>
+  </si>
+  <si>
+    <t>2004............................................................................. .</t>
+  </si>
+  <si>
+    <t>2005............................................................................. .</t>
+  </si>
+  <si>
+    <t>2006............................................................................. .</t>
+  </si>
+  <si>
+    <t>2007............................................................................. .</t>
+  </si>
+  <si>
+    <t>2008............................................................................. .</t>
+  </si>
+  <si>
+    <t>2009............................................................................. .</t>
+  </si>
+  <si>
+    <t>2010............................................................................. .</t>
+  </si>
+  <si>
+    <t>2011............................................................................. .</t>
+  </si>
+  <si>
+    <t>2012............................................................................. .</t>
+  </si>
+  <si>
+    <t>2013............................................................................. .</t>
+  </si>
+  <si>
+    <t>2014............................................................................. .</t>
+  </si>
+  <si>
+    <t>2015............................................................................. .</t>
+  </si>
+  <si>
+    <t>2016............................................................................. .</t>
+  </si>
+  <si>
+    <t>2017............................................................................. .</t>
+  </si>
+  <si>
+    <t>2018............................................................................. .</t>
+  </si>
+  <si>
+    <t>2019............................................................................. .</t>
+  </si>
+  <si>
+    <t>2020............................................................................. .</t>
+  </si>
+  <si>
+    <t>2021............................................................................. .</t>
+  </si>
+  <si>
+    <t>2022............................................................................. .</t>
+  </si>
+  <si>
+    <t>2023............................................................................. .</t>
+  </si>
+  <si>
+    <t>2024............................................................................. .</t>
+  </si>
+  <si>
+    <t>https://farmdocdaily.illinois.edu/2025/10/large-increase-in-machinery-costs-suggests-need-to-reconsider-machinery-purchase-decisions.html?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>CPI</t>
+  </si>
+  <si>
+    <t>CPI indexed to 2000</t>
+  </si>
+  <si>
+    <t>Nominal tractor price index</t>
+  </si>
+  <si>
+    <t>Real tractor price index</t>
+  </si>
+  <si>
+    <t>Real annual price growth:</t>
+  </si>
+  <si>
+    <t>per year</t>
+  </si>
+  <si>
+    <t>Table 5. Regression model comparison</t>
+  </si>
+  <si>
+    <t>Average hp.hr/gal</t>
+  </si>
+  <si>
+    <t>tested tractors</t>
+  </si>
+  <si>
+    <t>year coefficient</t>
+  </si>
+  <si>
+    <t>avg %chg in hp.hr/gal per year</t>
+  </si>
+  <si>
+    <t>Model 1: 1987-2021</t>
+  </si>
+  <si>
+    <t>Model 2</t>
+  </si>
+  <si>
+    <t>Model 3: Tier 4 only (2015-21)</t>
+  </si>
+  <si>
+    <t>Elasticity: Δprice/Δeff</t>
+  </si>
+  <si>
+    <t>Average elasticity:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="#0.0"/>
+    <numFmt numFmtId="172" formatCode="#0.000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1756,6 +2030,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1808,7 +2088,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1854,6 +2134,19 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5126,6 +5419,72 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>573315</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Line graph showing U.S. Tractor Prices Paid Index from 2000 to 2024. The index starts at 68 in 2000 and rises to 70 in 2002, 76 in 2005, 82 in 2007, 91 in 2009, 100 in 2011, 106 in 2013, 110 in 2015, and 113 in 2017. The index dips slightly to 112 in 2018, then rises to 123 in 2021, followed by sharp increases to 138 in 2023 and 139 in 2024. The trend shows generally steady growth with a notable dip in 2018 and particularly steep increases after 2020. Source: USDA, NASS.">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{51158697-A946-42D5-B1A2-8CA2048C4379}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="3048000"/>
+          <a:ext cx="8315779" cy="4657725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -5443,7 +5802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6F6B216-0153-49F1-A327-FA35702ED267}">
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="60.42578125" customWidth="1"/>
@@ -5689,52 +6048,77 @@
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="B57" s="15" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B58" s="2">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5745,6 +6129,916 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1873BFA-BFB8-479B-8580-77E23D72D642}">
+  <dimension ref="B1:M51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" t="s">
+        <v>116</v>
+      </c>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C4" s="12">
+        <v>0.8</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11">
+        <f>D4+$E$6</f>
+        <v>6928</v>
+      </c>
+      <c r="L4" t="s">
+        <v>117</v>
+      </c>
+      <c r="M4" s="1">
+        <f>AVERAGE(H5:H11)</f>
+        <v>7.5361437213570515</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C5" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="D5" s="11">
+        <v>472</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" ref="F5:F11" si="0">D5+$E$6</f>
+        <v>7400</v>
+      </c>
+      <c r="H5">
+        <f>((F5-$F$4)/($F$4))/((C5-$C$4)/($C$4))</f>
+        <v>5.4503464203233207</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="L5" t="s">
+        <v>118</v>
+      </c>
+      <c r="M5" s="1">
+        <f>AVERAGE(H13:H17)</f>
+        <v>10.236696165191734</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="12">
+        <v>0.82</v>
+      </c>
+      <c r="D6">
+        <v>977</v>
+      </c>
+      <c r="E6" s="11">
+        <v>6928</v>
+      </c>
+      <c r="F6" s="11">
+        <f t="shared" si="0"/>
+        <v>7905</v>
+      </c>
+      <c r="H6">
+        <f t="shared" ref="H6:H11" si="1">((F6-$F$4)/($F$4))/((C6-$C$4)/($C$4))</f>
+        <v>5.6408775981524517</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="L6" t="s">
+        <v>119</v>
+      </c>
+      <c r="M6" s="1">
+        <f>AVERAGE(H19:H24)</f>
+        <v>7.5709278650378069</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C7" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D7" s="11">
+        <v>2759</v>
+      </c>
+      <c r="F7" s="11">
+        <f t="shared" si="0"/>
+        <v>9687</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>7.9647806004619088</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="L7" t="s">
+        <v>120</v>
+      </c>
+      <c r="M7" s="1">
+        <f>AVERAGE(H26:H29)</f>
+        <v>13.093142804855722</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C8" s="12">
+        <v>0.85</v>
+      </c>
+      <c r="D8">
+        <v>3561</v>
+      </c>
+      <c r="F8" s="11">
+        <f t="shared" si="0"/>
+        <v>10489</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>8.2240184757505883</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="L8" t="s">
+        <v>121</v>
+      </c>
+      <c r="M8" s="1">
+        <f>AVERAGE(H31:H35)</f>
+        <v>6.8445086849877326</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C9" s="12">
+        <v>0.93</v>
+      </c>
+      <c r="D9" s="11">
+        <v>10027</v>
+      </c>
+      <c r="F9" s="11">
+        <f t="shared" si="0"/>
+        <v>16955</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>8.9065553384260081</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="L9" t="s">
+        <v>122</v>
+      </c>
+      <c r="M9" s="1">
+        <f>AVERAGE(H37:H42)</f>
+        <v>4.7753002649653098</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C10" s="12">
+        <v>0.95</v>
+      </c>
+      <c r="D10" s="11">
+        <v>10494</v>
+      </c>
+      <c r="F10" s="11">
+        <f t="shared" si="0"/>
+        <v>17422</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>8.0785219399538146</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="L10" t="s">
+        <v>123</v>
+      </c>
+      <c r="M10" s="1">
+        <f>AVERAGE(H44:H46)</f>
+        <v>10.329147244310422</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C11" s="12">
+        <v>0.99</v>
+      </c>
+      <c r="D11" s="11">
+        <v>13966</v>
+      </c>
+      <c r="F11" s="11">
+        <f t="shared" si="0"/>
+        <v>20894</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="1"/>
+        <v>8.4879056764312661</v>
+      </c>
+      <c r="I11" s="1"/>
+      <c r="L11" t="s">
+        <v>124</v>
+      </c>
+      <c r="M11" s="1">
+        <f>AVERAGE(H48:H50)</f>
+        <v>7.1185033686236947</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C12" s="12">
+        <v>0.82</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11">
+        <f>D12+$E$14</f>
+        <v>21244</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C13" s="12">
+        <v>0.83</v>
+      </c>
+      <c r="D13" s="11">
+        <v>2534</v>
+      </c>
+      <c r="F13" s="11">
+        <f t="shared" ref="F13:F17" si="2">D13+$E$14</f>
+        <v>23778</v>
+      </c>
+      <c r="H13">
+        <f>((F13-$F$12)/($F$12))/((C13-$C$12)/($C$12))</f>
+        <v>9.7810205234419048</v>
+      </c>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D14" s="5">
+        <v>5370</v>
+      </c>
+      <c r="E14" s="11">
+        <v>21244</v>
+      </c>
+      <c r="F14" s="11">
+        <f t="shared" si="2"/>
+        <v>26614</v>
+      </c>
+      <c r="H14">
+        <f t="shared" ref="H14:H17" si="3">((F14-$F$12)/($F$12))/((C14-$C$12)/($C$12))</f>
+        <v>10.363867444925617</v>
+      </c>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C15" s="12">
+        <v>0.85</v>
+      </c>
+      <c r="D15" s="11">
+        <v>8544</v>
+      </c>
+      <c r="F15" s="11">
+        <f t="shared" si="2"/>
+        <v>29788</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="3"/>
+        <v>10.993033327057042</v>
+      </c>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C16" s="12">
+        <v>0.94</v>
+      </c>
+      <c r="D16" s="11">
+        <v>32796</v>
+      </c>
+      <c r="F16" s="11">
+        <f t="shared" si="2"/>
+        <v>54040</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="3"/>
+        <v>10.549143287516475</v>
+      </c>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C17" s="12">
+        <v>0.97</v>
+      </c>
+      <c r="D17" s="11">
+        <v>36904</v>
+      </c>
+      <c r="F17" s="11">
+        <f t="shared" si="2"/>
+        <v>58148</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="3"/>
+        <v>9.4964162430176344</v>
+      </c>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C18" s="12">
+        <v>0.82</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="F18" s="11">
+        <f>D18+$E$21</f>
+        <v>8404</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C19" s="12">
+        <v>0.83</v>
+      </c>
+      <c r="D19" s="11">
+        <v>634</v>
+      </c>
+      <c r="F19" s="11">
+        <f t="shared" ref="F19:F24" si="4">D19+$E$21</f>
+        <v>9038</v>
+      </c>
+      <c r="H19">
+        <f>((F19-$F$18)/($F$18))/((C19-$C$18)/($C$18))</f>
+        <v>6.1861018562589187</v>
+      </c>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D20">
+        <v>1315</v>
+      </c>
+      <c r="F20" s="11">
+        <f t="shared" si="4"/>
+        <v>9719</v>
+      </c>
+      <c r="H20">
+        <f t="shared" ref="H20:H24" si="5">((F20-$F$18)/($F$18))/((C20-$C$18)/($C$18))</f>
+        <v>6.4153974297953296</v>
+      </c>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="12">
+        <v>0.85</v>
+      </c>
+      <c r="D21" s="11">
+        <v>2048</v>
+      </c>
+      <c r="E21" s="11">
+        <v>8404</v>
+      </c>
+      <c r="F21" s="11">
+        <f t="shared" si="4"/>
+        <v>10452</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="5"/>
+        <v>6.6609551007456709</v>
+      </c>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C22" s="12">
+        <v>0.87</v>
+      </c>
+      <c r="D22">
+        <v>3683</v>
+      </c>
+      <c r="F22" s="11">
+        <f t="shared" si="4"/>
+        <v>12087</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="5"/>
+        <v>7.1871965730604401</v>
+      </c>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="12">
+        <v>0.88</v>
+      </c>
+      <c r="D23" s="11">
+        <v>4594</v>
+      </c>
+      <c r="F23" s="11">
+        <f t="shared" si="4"/>
+        <v>12998</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="5"/>
+        <v>7.4708075519593775</v>
+      </c>
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C24" s="12">
+        <v>0.97</v>
+      </c>
+      <c r="D24" s="5">
+        <v>17687</v>
+      </c>
+      <c r="F24" s="11">
+        <f t="shared" si="4"/>
+        <v>26091</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="5"/>
+        <v>11.505108678407106</v>
+      </c>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="11">
+        <f>D25+$E$27</f>
+        <v>18915</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C26" s="12">
+        <v>0.86</v>
+      </c>
+      <c r="D26" s="11">
+        <v>4785</v>
+      </c>
+      <c r="F26" s="11">
+        <f t="shared" ref="F26:F29" si="6">D26+$E$27</f>
+        <v>23700</v>
+      </c>
+      <c r="H26">
+        <f>((F26-$F$25)/($F$25))/((C26-$C$25)/($C$25))</f>
+        <v>10.624900872323542</v>
+      </c>
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>120</v>
+      </c>
+      <c r="C27" s="12">
+        <v>0.88</v>
+      </c>
+      <c r="D27" s="11">
+        <v>10781</v>
+      </c>
+      <c r="E27" s="11">
+        <v>18915</v>
+      </c>
+      <c r="F27" s="11">
+        <f t="shared" si="6"/>
+        <v>29696</v>
+      </c>
+      <c r="H27">
+        <f t="shared" ref="H27:H29" si="7">((F27-$F$25)/($F$25))/((C27-$C$25)/($C$25))</f>
+        <v>11.969389373513073</v>
+      </c>
+      <c r="I27" s="1"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="12">
+        <v>0.89</v>
+      </c>
+      <c r="D28" s="11">
+        <v>14326</v>
+      </c>
+      <c r="F28" s="11">
+        <f t="shared" si="6"/>
+        <v>33241</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="7"/>
+        <v>12.724123711340194</v>
+      </c>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C29" s="12">
+        <v>0.97</v>
+      </c>
+      <c r="D29" s="5">
+        <v>49923</v>
+      </c>
+      <c r="F29" s="11">
+        <f t="shared" si="6"/>
+        <v>68838</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="7"/>
+        <v>17.054157262246079</v>
+      </c>
+      <c r="I29" s="1"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="12">
+        <v>0.77</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="F30" s="11">
+        <f>D30+$E$32</f>
+        <v>6659</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C31" s="12">
+        <v>0.78</v>
+      </c>
+      <c r="D31" s="11">
+        <v>540</v>
+      </c>
+      <c r="F31" s="11">
+        <f t="shared" ref="F31:F35" si="8">D31+$E$32</f>
+        <v>7199</v>
+      </c>
+      <c r="H31">
+        <f>((F31-$F$30)/($F$30))/((C31-$C$30)/($C$30))</f>
+        <v>6.244180807929113</v>
+      </c>
+      <c r="I31" s="1"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" s="12">
+        <v>0.79</v>
+      </c>
+      <c r="D32" s="5">
+        <v>1124</v>
+      </c>
+      <c r="E32" s="11">
+        <v>6659</v>
+      </c>
+      <c r="F32" s="11">
+        <f t="shared" si="8"/>
+        <v>7783</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H35" si="9">((F32-$F$30)/($F$30))/((C32-$C$30)/($C$30))</f>
+        <v>6.4985733593632622</v>
+      </c>
+      <c r="I32" s="1"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C33" s="12">
+        <v>0.8</v>
+      </c>
+      <c r="D33" s="11">
+        <v>1756</v>
+      </c>
+      <c r="F33" s="11">
+        <f t="shared" si="8"/>
+        <v>8415</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="9"/>
+        <v>6.7683836411873592</v>
+      </c>
+      <c r="I33" s="1"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C34" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="D34" s="5">
+        <v>2439</v>
+      </c>
+      <c r="F34" s="11">
+        <f t="shared" si="8"/>
+        <v>9098</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="9"/>
+        <v>7.0507208289532901</v>
+      </c>
+      <c r="I34" s="1"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C35" s="12">
+        <v>0.83</v>
+      </c>
+      <c r="D35" s="11">
+        <v>3975</v>
+      </c>
+      <c r="F35" s="11">
+        <f t="shared" si="8"/>
+        <v>10634</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="9"/>
+        <v>7.6606847875056383</v>
+      </c>
+      <c r="I35" s="1"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C36" s="12">
+        <v>0.77</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="F36" s="11">
+        <f>D36+$E$39</f>
+        <v>19122</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C37" s="12">
+        <v>0.78</v>
+      </c>
+      <c r="D37" s="5">
+        <v>1097</v>
+      </c>
+      <c r="F37" s="11">
+        <f t="shared" ref="F37:F42" si="10">D37+$E$39</f>
+        <v>20219</v>
+      </c>
+      <c r="H37">
+        <f>((F37-$F$36)/($F$36))/((C37-$C$36)/($C$36))</f>
+        <v>4.4173726597636191</v>
+      </c>
+      <c r="I37" s="1"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C38" s="12">
+        <v>0.79</v>
+      </c>
+      <c r="D38" s="5">
+        <v>2256</v>
+      </c>
+      <c r="F38" s="11">
+        <f t="shared" si="10"/>
+        <v>21378</v>
+      </c>
+      <c r="H38">
+        <f t="shared" ref="H38:H42" si="11">((F38-$F$36)/($F$36))/((C38-$C$36)/($C$36))</f>
+        <v>4.5422026984624999</v>
+      </c>
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="12">
+        <v>0.8</v>
+      </c>
+      <c r="D39" s="5">
+        <v>3483</v>
+      </c>
+      <c r="E39" s="11">
+        <v>19122</v>
+      </c>
+      <c r="F39" s="11">
+        <f t="shared" si="10"/>
+        <v>22605</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="11"/>
+        <v>4.67508628804518</v>
+      </c>
+      <c r="I39" s="1"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C40" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="D40">
+        <v>4779</v>
+      </c>
+      <c r="F40" s="11">
+        <f t="shared" si="10"/>
+        <v>23901</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="11"/>
+        <v>4.8109899592092837</v>
+      </c>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C41" s="12">
+        <v>0.82</v>
+      </c>
+      <c r="D41" s="11">
+        <v>6150</v>
+      </c>
+      <c r="F41" s="11">
+        <f t="shared" si="10"/>
+        <v>25272</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="11"/>
+        <v>4.9529337935362481</v>
+      </c>
+      <c r="I41" s="1"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C42" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D42">
+        <v>9132</v>
+      </c>
+      <c r="F42" s="11">
+        <f t="shared" si="10"/>
+        <v>28254</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="11"/>
+        <v>5.2532161907750279</v>
+      </c>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C43" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="F43" s="11">
+        <f>D43+$E$44</f>
+        <v>7294</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>123</v>
+      </c>
+      <c r="C44" s="12">
+        <v>0.83</v>
+      </c>
+      <c r="D44" s="5">
+        <v>1722</v>
+      </c>
+      <c r="E44" s="11">
+        <v>7294</v>
+      </c>
+      <c r="F44" s="11">
+        <f t="shared" ref="F44:F46" si="12">D44+$E$44</f>
+        <v>9016</v>
+      </c>
+      <c r="H44">
+        <f>((F44-$F$43)/($F$43))/((C44-$C$43)/($C$43))</f>
+        <v>9.5614203454894877</v>
+      </c>
+      <c r="I44" s="1"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C45" s="12">
+        <v>0.84</v>
+      </c>
+      <c r="D45">
+        <v>2730</v>
+      </c>
+      <c r="F45" s="11">
+        <f t="shared" si="12"/>
+        <v>10024</v>
+      </c>
+      <c r="H45">
+        <f t="shared" ref="H45:H46" si="13">((F45-$F$43)/($F$43))/((C45-$C$43)/($C$43))</f>
+        <v>10.10556621881001</v>
+      </c>
+      <c r="I45" s="1"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C46" s="12">
+        <v>0.86</v>
+      </c>
+      <c r="D46" s="11">
+        <v>5097</v>
+      </c>
+      <c r="F46" s="11">
+        <f t="shared" si="12"/>
+        <v>12391</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="13"/>
+        <v>11.320455168631767</v>
+      </c>
+      <c r="I46" s="1"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C47" s="12">
+        <v>0.81</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="F47" s="11">
+        <f>D47+$E$48</f>
+        <v>18702</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="12">
+        <v>0.83</v>
+      </c>
+      <c r="D48" s="11">
+        <v>3071</v>
+      </c>
+      <c r="E48" s="11">
+        <v>18702</v>
+      </c>
+      <c r="F48" s="11">
+        <f t="shared" ref="F48:F50" si="14">D48+$E$48</f>
+        <v>21773</v>
+      </c>
+      <c r="H48">
+        <f>((F48-$F$47)/($F$47))/((C48-$C$47)/($C$47))</f>
+        <v>6.6503849855630728</v>
+      </c>
+      <c r="I48" s="1"/>
+    </row>
+    <row r="49" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C49" s="12">
+        <v>0.85</v>
+      </c>
+      <c r="D49" s="11">
+        <v>6521</v>
+      </c>
+      <c r="F49" s="11">
+        <f t="shared" si="14"/>
+        <v>25223</v>
+      </c>
+      <c r="H49">
+        <f t="shared" ref="H49:H50" si="15">((F49-$F$47)/($F$47))/((C49-$C$47)/($C$47))</f>
+        <v>7.060755534167483</v>
+      </c>
+      <c r="I49" s="1"/>
+    </row>
+    <row r="50" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C50" s="12">
+        <v>0.87</v>
+      </c>
+      <c r="D50" s="11">
+        <v>10590</v>
+      </c>
+      <c r="F50" s="11">
+        <f t="shared" si="14"/>
+        <v>29292</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="15"/>
+        <v>7.6443695861405265</v>
+      </c>
+      <c r="I50" s="1"/>
+    </row>
+    <row r="51" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="I51" s="13">
+        <f>AVERAGE(H1:H50)</f>
+        <v>8.126972362529246</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D39F440-FA8D-440E-B9E0-04BD2776E781}">
   <dimension ref="B2:O26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6560,7 +7854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75FF9701-D73C-4593-9C81-F6045C33961E}">
   <dimension ref="A1:AD94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7944,7 +9238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1011C56E-59CC-41D7-BD37-B8D3833EEA91}">
   <dimension ref="B2:G36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8484,7 +9778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFF80A1E-9380-4D67-8452-F9501E3A0DC6}">
   <dimension ref="A2:J19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8827,7 +10121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8718AA-AC7D-4D9E-9BAB-C38A4CE85A96}">
   <dimension ref="A1:W63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10117,7 +11411,258 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6BD96FA-EB4C-4695-AB05-D346A69359A2}">
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.5703125" customWidth="1"/>
+    <col min="2" max="4" width="10.7109375" customWidth="1"/>
+    <col min="20" max="20" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="6.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="B4" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>606</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>607</v>
+      </c>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>601</v>
+      </c>
+      <c r="B5">
+        <v>17.670000000000002</v>
+      </c>
+      <c r="C5">
+        <v>17.64</v>
+      </c>
+      <c r="D5">
+        <v>18.37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>602</v>
+      </c>
+      <c r="B6">
+        <v>1440</v>
+      </c>
+      <c r="C6">
+        <v>1297</v>
+      </c>
+      <c r="D6">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>603</v>
+      </c>
+      <c r="B7">
+        <v>9.7000000000000003E-2</v>
+      </c>
+      <c r="C7">
+        <v>0.105</v>
+      </c>
+      <c r="D7">
+        <v>0.14099999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>604</v>
+      </c>
+      <c r="B8" s="9">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="C8" s="9">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="D8" s="9">
+        <v>7.7000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>2001</v>
+      </c>
+      <c r="C38">
+        <v>2011</v>
+      </c>
+      <c r="D38">
+        <v>2021</v>
+      </c>
+      <c r="F38">
+        <v>2015</v>
+      </c>
+      <c r="G38">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>596</v>
+      </c>
+      <c r="B39">
+        <v>68</v>
+      </c>
+      <c r="C39">
+        <v>100</v>
+      </c>
+      <c r="D39">
+        <v>123</v>
+      </c>
+      <c r="F39">
+        <v>110</v>
+      </c>
+      <c r="G39">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>594</v>
+      </c>
+      <c r="B40">
+        <f>cpi!D39</f>
+        <v>177.1</v>
+      </c>
+      <c r="C40">
+        <f>cpi!D49</f>
+        <v>224.93899999999999</v>
+      </c>
+      <c r="D40">
+        <f>cpi!D59</f>
+        <v>270.97000000000003</v>
+      </c>
+      <c r="F40">
+        <f>cpi!D53</f>
+        <v>237.017</v>
+      </c>
+      <c r="G40">
+        <f>cpi!D59</f>
+        <v>270.97000000000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>595</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41">
+        <f>C40/B40</f>
+        <v>1.2701242236024846</v>
+      </c>
+      <c r="D41">
+        <f>D40/B40</f>
+        <v>1.5300395256916999</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <f>G40/F40</f>
+        <v>1.143251327963817</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>597</v>
+      </c>
+      <c r="B42">
+        <f>B39/B41</f>
+        <v>68</v>
+      </c>
+      <c r="C42">
+        <f>C39/C41</f>
+        <v>78.732456354833971</v>
+      </c>
+      <c r="D42">
+        <f>D39/D41</f>
+        <v>80.390080082665961</v>
+      </c>
+      <c r="F42">
+        <f t="shared" ref="F42:G42" si="0">F39/F41</f>
+        <v>110</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="0"/>
+        <v>114.58547809720632</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>598</v>
+      </c>
+      <c r="B44" s="39">
+        <f>(D42/B42)^(1/(D38-B38))-1</f>
+        <v>8.4042733414155801E-3</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="F44" s="39">
+        <f>(G42/F42)^(1/(G38-F38))-1</f>
+        <v>6.8300041962665592E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>608</v>
+      </c>
+      <c r="B47" s="7">
+        <f>B44/B8</f>
+        <v>1.5280496984391965</v>
+      </c>
+      <c r="F47" s="7">
+        <f>F44/D8</f>
+        <v>0.88701353198266997</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>609</v>
+      </c>
+      <c r="B49" s="7">
+        <f>AVERAGE(B47,F47)</f>
+        <v>1.2075316152109332</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D5271D-8741-40B6-92F2-97D4F5B6382F}">
   <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10202,9 +11747,9 @@
         <f>Lighting!G63</f>
         <v>1.1617489485420724</v>
       </c>
-      <c r="K2" s="27">
-        <f>H2</f>
-        <v>3.1863586362595919</v>
+      <c r="K2" s="26">
+        <f>mobile!$B$49</f>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -10248,8 +11793,8 @@
         <v>1.1617489485420724</v>
       </c>
       <c r="K3" s="27">
-        <f t="shared" ref="K3:K13" si="3">H3</f>
-        <v>3.1863586362595919</v>
+        <f>$K$2</f>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -10265,7 +11810,7 @@
         <v>5.8575070498108852</v>
       </c>
       <c r="D4" s="27">
-        <f t="shared" ref="D4:D13" si="4">C4</f>
+        <f t="shared" ref="D4:D13" si="3">C4</f>
         <v>5.8575070498108852</v>
       </c>
       <c r="E4" s="27">
@@ -10273,11 +11818,11 @@
         <v>5.8575070498108852</v>
       </c>
       <c r="F4" s="27">
-        <f t="shared" ref="F4:F13" si="5">$F$2</f>
+        <f t="shared" ref="F4:F13" si="4">$F$2</f>
         <v>0.84489777592279791</v>
       </c>
       <c r="G4" s="27">
-        <f t="shared" ref="G4:G13" si="6">$G$2</f>
+        <f t="shared" ref="G4:G13" si="5">$G$2</f>
         <v>2.5525704426134292</v>
       </c>
       <c r="H4" s="27">
@@ -10289,12 +11834,12 @@
         <v>7.4277116196437323</v>
       </c>
       <c r="J4" s="27">
-        <f t="shared" ref="J4:J13" si="7">$J$2</f>
+        <f t="shared" ref="J4:J13" si="6">$J$2</f>
         <v>1.1617489485420724</v>
       </c>
       <c r="K4" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <f t="shared" ref="K4:K13" si="7">$K$2</f>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -10310,7 +11855,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D5" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E5" s="27">
@@ -10318,11 +11863,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F5" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G5" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G5" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H5" s="27">
@@ -10334,12 +11879,12 @@
         <v>2.4280165739690442</v>
       </c>
       <c r="J5" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K5" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K5" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -10355,7 +11900,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D6" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E6" s="27">
@@ -10363,11 +11908,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F6" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G6" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G6" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H6" s="27">
@@ -10375,16 +11920,16 @@
         <v>3.1863586362595919</v>
       </c>
       <c r="I6" s="27">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(B6:C6)</f>
         <v>6.4699072941282818</v>
       </c>
       <c r="J6" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K6" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K6" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -10408,11 +11953,11 @@
         <v>4.0277954796628537</v>
       </c>
       <c r="F7" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G7" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G7" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H7" s="27">
@@ -10424,12 +11969,12 @@
         <v>5.110100116295146</v>
       </c>
       <c r="J7" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K7" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K7" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -10445,7 +11990,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D8" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E8" s="27">
@@ -10453,11 +11998,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F8" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G8" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G8" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H8" s="27">
@@ -10469,12 +12014,12 @@
         <v>6.4699072941282818</v>
       </c>
       <c r="J8" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K8" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K8" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -10490,7 +12035,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D9" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E9" s="27">
@@ -10498,11 +12043,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F9" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G9" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G9" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H9" s="27">
@@ -10514,12 +12059,12 @@
         <v>6.4699072941282818</v>
       </c>
       <c r="J9" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K9" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K9" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -10535,7 +12080,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D10" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E10" s="27">
@@ -10543,11 +12088,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F10" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G10" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G10" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H10" s="27">
@@ -10559,12 +12104,12 @@
         <v>5.5980000494957007</v>
       </c>
       <c r="J10" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K10" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K10" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -10580,7 +12125,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D11" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E11" s="27">
@@ -10588,11 +12133,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F11" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G11" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G11" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H11" s="27">
@@ -10604,12 +12149,12 @@
         <v>5.5980000494957007</v>
       </c>
       <c r="J11" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K11" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K11" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -10625,7 +12170,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D12" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E12" s="27">
@@ -10633,11 +12178,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F12" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G12" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G12" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H12" s="27">
@@ -10649,12 +12194,12 @@
         <v>5.5980000494957007</v>
       </c>
       <c r="J12" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K12" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K12" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -10670,7 +12215,7 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="D13" s="27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.1980839095148221</v>
       </c>
       <c r="E13" s="27">
@@ -10678,11 +12223,11 @@
         <v>2.1980839095148221</v>
       </c>
       <c r="F13" s="27">
+        <f t="shared" si="4"/>
+        <v>0.84489777592279791</v>
+      </c>
+      <c r="G13" s="27">
         <f t="shared" si="5"/>
-        <v>0.84489777592279791</v>
-      </c>
-      <c r="G13" s="27">
-        <f t="shared" si="6"/>
         <v>2.5525704426134292</v>
       </c>
       <c r="H13" s="27">
@@ -10694,12 +12239,12 @@
         <v>5.5980000494957007</v>
       </c>
       <c r="J13" s="27">
+        <f t="shared" si="6"/>
+        <v>1.1617489485420724</v>
+      </c>
+      <c r="K13" s="27">
         <f t="shared" si="7"/>
-        <v>1.1617489485420724</v>
-      </c>
-      <c r="K13" s="27">
-        <f t="shared" si="3"/>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
   </sheetData>
@@ -10707,7 +12252,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BB977EF-DFFE-4EEF-A0E1-DBBDDDFA9996}">
   <sheetPr>
     <tabColor theme="3" tint="9.9978637043366805E-2"/>
@@ -10796,8 +12341,8 @@
         <v>1.1617489485420724</v>
       </c>
       <c r="K2" s="27">
-        <f>calcs!K2</f>
-        <v>3.1863586362595919</v>
+        <f>mobile!B49</f>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -10842,7 +12387,7 @@
       </c>
       <c r="K3" s="27">
         <f>calcs!K3</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -10887,7 +12432,7 @@
       </c>
       <c r="K4" s="27">
         <f>calcs!K4</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -10932,7 +12477,7 @@
       </c>
       <c r="K5" s="27">
         <f>calcs!K5</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -10977,7 +12522,7 @@
       </c>
       <c r="K6" s="27">
         <f>calcs!K6</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -11022,7 +12567,7 @@
       </c>
       <c r="K7" s="27">
         <f>calcs!K7</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -11067,7 +12612,7 @@
       </c>
       <c r="K8" s="27">
         <f>calcs!K8</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -11112,7 +12657,7 @@
       </c>
       <c r="K9" s="27">
         <f>calcs!K9</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -11157,7 +12702,7 @@
       </c>
       <c r="K10" s="27">
         <f>calcs!K10</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -11202,7 +12747,7 @@
       </c>
       <c r="K11" s="27">
         <f>calcs!K11</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -11247,7 +12792,7 @@
       </c>
       <c r="K12" s="27">
         <f>calcs!K12</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -11292,7 +12837,7 @@
       </c>
       <c r="K13" s="27">
         <f>calcs!K13</f>
-        <v>3.1863586362595919</v>
+        <v>1.2075316152109332</v>
       </c>
     </row>
   </sheetData>
@@ -11313,6 +12858,1419 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D47034FE-671A-414C-B645-6D2F26709972}">
+  <dimension ref="A1:O62"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="14" max="14" width="10.5703125" customWidth="1"/>
+    <col min="15" max="15" width="28.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>527</v>
+      </c>
+      <c r="B4" t="s">
+        <v>528</v>
+      </c>
+      <c r="D4" t="s">
+        <v>529</v>
+      </c>
+      <c r="E4" t="s">
+        <v>530</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>532</v>
+      </c>
+      <c r="C5" t="s">
+        <v>533</v>
+      </c>
+      <c r="E5" t="s">
+        <v>534</v>
+      </c>
+      <c r="F5" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>535</v>
+      </c>
+      <c r="B6" t="s">
+        <v>536</v>
+      </c>
+      <c r="C6" t="s">
+        <v>536</v>
+      </c>
+      <c r="D6">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="E6">
+        <v>4.7</v>
+      </c>
+      <c r="F6">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>537</v>
+      </c>
+      <c r="B7" t="s">
+        <v>536</v>
+      </c>
+      <c r="C7" t="s">
+        <v>536</v>
+      </c>
+      <c r="D7">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="E7">
+        <v>6.2</v>
+      </c>
+      <c r="F7">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>538</v>
+      </c>
+      <c r="B8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C8" t="s">
+        <v>536</v>
+      </c>
+      <c r="D8">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="E8">
+        <v>5.6</v>
+      </c>
+      <c r="F8">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>539</v>
+      </c>
+      <c r="B9" t="s">
+        <v>536</v>
+      </c>
+      <c r="C9" t="s">
+        <v>536</v>
+      </c>
+      <c r="D9">
+        <v>40.5</v>
+      </c>
+      <c r="E9">
+        <v>3.3</v>
+      </c>
+      <c r="F9">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>540</v>
+      </c>
+      <c r="B10" t="s">
+        <v>536</v>
+      </c>
+      <c r="C10" t="s">
+        <v>536</v>
+      </c>
+      <c r="D10">
+        <v>41.8</v>
+      </c>
+      <c r="E10">
+        <v>3.4</v>
+      </c>
+      <c r="F10">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>541</v>
+      </c>
+      <c r="B11" t="s">
+        <v>536</v>
+      </c>
+      <c r="C11" t="s">
+        <v>536</v>
+      </c>
+      <c r="D11">
+        <v>44.4</v>
+      </c>
+      <c r="E11">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="F11">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>542</v>
+      </c>
+      <c r="B12" t="s">
+        <v>536</v>
+      </c>
+      <c r="C12" t="s">
+        <v>536</v>
+      </c>
+      <c r="D12">
+        <v>49.3</v>
+      </c>
+      <c r="E12">
+        <v>12.3</v>
+      </c>
+      <c r="F12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>543</v>
+      </c>
+      <c r="B13" t="s">
+        <v>536</v>
+      </c>
+      <c r="C13" t="s">
+        <v>536</v>
+      </c>
+      <c r="D13">
+        <v>53.8</v>
+      </c>
+      <c r="E13">
+        <v>6.9</v>
+      </c>
+      <c r="F13">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B14" t="s">
+        <v>536</v>
+      </c>
+      <c r="C14" t="s">
+        <v>536</v>
+      </c>
+      <c r="D14">
+        <v>56.9</v>
+      </c>
+      <c r="E14">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="F14">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>545</v>
+      </c>
+      <c r="B15" t="s">
+        <v>536</v>
+      </c>
+      <c r="C15" t="s">
+        <v>536</v>
+      </c>
+      <c r="D15">
+        <v>60.6</v>
+      </c>
+      <c r="E15">
+        <v>6.7</v>
+      </c>
+      <c r="F15">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>546</v>
+      </c>
+      <c r="B16" t="s">
+        <v>536</v>
+      </c>
+      <c r="C16" t="s">
+        <v>536</v>
+      </c>
+      <c r="D16">
+        <v>65.2</v>
+      </c>
+      <c r="E16">
+        <v>9</v>
+      </c>
+      <c r="F16">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>547</v>
+      </c>
+      <c r="B17" t="s">
+        <v>536</v>
+      </c>
+      <c r="C17" t="s">
+        <v>536</v>
+      </c>
+      <c r="D17">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="E17">
+        <v>13.3</v>
+      </c>
+      <c r="F17">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>548</v>
+      </c>
+      <c r="B18" t="s">
+        <v>536</v>
+      </c>
+      <c r="C18" t="s">
+        <v>536</v>
+      </c>
+      <c r="D18">
+        <v>82.4</v>
+      </c>
+      <c r="E18">
+        <v>12.5</v>
+      </c>
+      <c r="F18">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>549</v>
+      </c>
+      <c r="B19" t="s">
+        <v>536</v>
+      </c>
+      <c r="C19" t="s">
+        <v>536</v>
+      </c>
+      <c r="D19">
+        <v>90.9</v>
+      </c>
+      <c r="E19">
+        <v>8.9</v>
+      </c>
+      <c r="F19">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>550</v>
+      </c>
+      <c r="B20" t="s">
+        <v>536</v>
+      </c>
+      <c r="C20" t="s">
+        <v>536</v>
+      </c>
+      <c r="D20">
+        <v>96.5</v>
+      </c>
+      <c r="E20">
+        <v>3.8</v>
+      </c>
+      <c r="F20">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>551</v>
+      </c>
+      <c r="B21" t="s">
+        <v>536</v>
+      </c>
+      <c r="C21" t="s">
+        <v>536</v>
+      </c>
+      <c r="D21">
+        <v>99.6</v>
+      </c>
+      <c r="E21">
+        <v>3.8</v>
+      </c>
+      <c r="F21">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>552</v>
+      </c>
+      <c r="B22" s="35">
+        <v>102.9</v>
+      </c>
+      <c r="C22" s="35">
+        <v>104.9</v>
+      </c>
+      <c r="D22" s="35">
+        <v>103.9</v>
+      </c>
+      <c r="E22">
+        <v>3.9</v>
+      </c>
+      <c r="F22">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>553</v>
+      </c>
+      <c r="B23" s="35">
+        <v>106.6</v>
+      </c>
+      <c r="C23" s="35">
+        <v>108.5</v>
+      </c>
+      <c r="D23" s="35">
+        <v>107.6</v>
+      </c>
+      <c r="E23">
+        <v>3.8</v>
+      </c>
+      <c r="F23">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>554</v>
+      </c>
+      <c r="B24" s="35">
+        <v>109.1</v>
+      </c>
+      <c r="C24" s="35">
+        <v>110.1</v>
+      </c>
+      <c r="D24" s="35">
+        <v>109.6</v>
+      </c>
+      <c r="E24">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F24">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>555</v>
+      </c>
+      <c r="B25" s="35">
+        <v>112.4</v>
+      </c>
+      <c r="C25" s="35">
+        <v>114.9</v>
+      </c>
+      <c r="D25" s="35">
+        <v>113.6</v>
+      </c>
+      <c r="E25">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F25">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>556</v>
+      </c>
+      <c r="B26" s="35">
+        <v>116.8</v>
+      </c>
+      <c r="C26" s="35">
+        <v>119.7</v>
+      </c>
+      <c r="D26" s="35">
+        <v>118.3</v>
+      </c>
+      <c r="E26">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F26">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>557</v>
+      </c>
+      <c r="B27" s="35">
+        <v>122.7</v>
+      </c>
+      <c r="C27" s="35">
+        <v>125.3</v>
+      </c>
+      <c r="D27" s="35">
+        <v>124</v>
+      </c>
+      <c r="E27">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F27">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>558</v>
+      </c>
+      <c r="B28" s="35">
+        <v>128.69999999999999</v>
+      </c>
+      <c r="C28" s="35">
+        <v>132.6</v>
+      </c>
+      <c r="D28" s="35">
+        <v>130.69999999999999</v>
+      </c>
+      <c r="E28">
+        <v>6.1</v>
+      </c>
+      <c r="F28">
+        <v>5.4</v>
+      </c>
+      <c r="G28" s="27">
+        <f>$D$50/D28</f>
+        <v>1.7566488140780414</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>559</v>
+      </c>
+      <c r="B29" s="35">
+        <v>135.19999999999999</v>
+      </c>
+      <c r="C29" s="35">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="D29" s="35">
+        <v>136.19999999999999</v>
+      </c>
+      <c r="E29">
+        <v>3.1</v>
+      </c>
+      <c r="F29">
+        <v>4.2</v>
+      </c>
+      <c r="G29" s="27">
+        <f t="shared" ref="G29:G62" si="0">$D$50/D29</f>
+        <v>1.6857121879588841</v>
+      </c>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>560</v>
+      </c>
+      <c r="B30" s="35">
+        <v>139.19999999999999</v>
+      </c>
+      <c r="C30" s="35">
+        <v>141.4</v>
+      </c>
+      <c r="D30" s="35">
+        <v>140.30000000000001</v>
+      </c>
+      <c r="E30">
+        <v>2.9</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30" s="27">
+        <f t="shared" si="0"/>
+        <v>1.6364504632929435</v>
+      </c>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="36"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>561</v>
+      </c>
+      <c r="B31" s="35">
+        <v>143.69999999999999</v>
+      </c>
+      <c r="C31" s="35">
+        <v>145.30000000000001</v>
+      </c>
+      <c r="D31" s="35">
+        <v>144.5</v>
+      </c>
+      <c r="E31">
+        <v>2.7</v>
+      </c>
+      <c r="F31">
+        <v>3</v>
+      </c>
+      <c r="G31" s="27">
+        <f t="shared" si="0"/>
+        <v>1.5888858131487889</v>
+      </c>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="36"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>562</v>
+      </c>
+      <c r="B32" s="35">
+        <v>147.19999999999999</v>
+      </c>
+      <c r="C32" s="35">
+        <v>149.30000000000001</v>
+      </c>
+      <c r="D32" s="35">
+        <v>148.19999999999999</v>
+      </c>
+      <c r="E32">
+        <v>2.7</v>
+      </c>
+      <c r="F32">
+        <v>2.6</v>
+      </c>
+      <c r="G32" s="27">
+        <f t="shared" si="0"/>
+        <v>1.5492172739541161</v>
+      </c>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+      <c r="O32" s="36"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>563</v>
+      </c>
+      <c r="B33" s="35">
+        <v>151.5</v>
+      </c>
+      <c r="C33" s="35">
+        <v>153.19999999999999</v>
+      </c>
+      <c r="D33" s="35">
+        <v>152.4</v>
+      </c>
+      <c r="E33">
+        <v>2.5</v>
+      </c>
+      <c r="F33">
+        <v>2.8</v>
+      </c>
+      <c r="G33" s="27">
+        <f t="shared" si="0"/>
+        <v>1.5065223097112861</v>
+      </c>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+      <c r="O33" s="36"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>564</v>
+      </c>
+      <c r="B34" s="35">
+        <v>155.80000000000001</v>
+      </c>
+      <c r="C34" s="35">
+        <v>157.9</v>
+      </c>
+      <c r="D34" s="35">
+        <v>156.9</v>
+      </c>
+      <c r="E34">
+        <v>3.3</v>
+      </c>
+      <c r="F34">
+        <v>3</v>
+      </c>
+      <c r="G34" s="27">
+        <f t="shared" si="0"/>
+        <v>1.4633142128744423</v>
+      </c>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
+      <c r="O34" s="36"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>565</v>
+      </c>
+      <c r="B35" s="35">
+        <v>159.9</v>
+      </c>
+      <c r="C35" s="35">
+        <v>161.19999999999999</v>
+      </c>
+      <c r="D35" s="35">
+        <v>160.5</v>
+      </c>
+      <c r="E35">
+        <v>1.7</v>
+      </c>
+      <c r="F35">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G35" s="27">
+        <f t="shared" si="0"/>
+        <v>1.4304922118380061</v>
+      </c>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="36"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>566</v>
+      </c>
+      <c r="B36" s="35">
+        <v>162.30000000000001</v>
+      </c>
+      <c r="C36" s="35">
+        <v>163.69999999999999</v>
+      </c>
+      <c r="D36" s="35">
+        <v>163</v>
+      </c>
+      <c r="E36">
+        <v>1.6</v>
+      </c>
+      <c r="F36">
+        <v>1.6</v>
+      </c>
+      <c r="G36" s="27">
+        <f t="shared" si="0"/>
+        <v>1.4085521472392637</v>
+      </c>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="36"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>567</v>
+      </c>
+      <c r="B37" s="35">
+        <v>165.4</v>
+      </c>
+      <c r="C37" s="35">
+        <v>167.8</v>
+      </c>
+      <c r="D37" s="35">
+        <v>166.6</v>
+      </c>
+      <c r="E37">
+        <v>2.7</v>
+      </c>
+      <c r="F37">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G37" s="27">
+        <f t="shared" si="0"/>
+        <v>1.3781152460984394</v>
+      </c>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="36"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>568</v>
+      </c>
+      <c r="B38" s="35">
+        <v>170.8</v>
+      </c>
+      <c r="C38" s="35">
+        <v>173.6</v>
+      </c>
+      <c r="D38" s="35">
+        <v>172.2</v>
+      </c>
+      <c r="E38">
+        <v>3.4</v>
+      </c>
+      <c r="F38">
+        <v>3.4</v>
+      </c>
+      <c r="G38" s="27">
+        <f t="shared" si="0"/>
+        <v>1.3332984901277585</v>
+      </c>
+      <c r="M38" s="2"/>
+      <c r="N38" s="37"/>
+      <c r="O38" s="36"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>569</v>
+      </c>
+      <c r="B39" s="35">
+        <v>176.6</v>
+      </c>
+      <c r="C39" s="35">
+        <v>177.5</v>
+      </c>
+      <c r="D39" s="35">
+        <v>177.1</v>
+      </c>
+      <c r="E39">
+        <v>1.6</v>
+      </c>
+      <c r="F39">
+        <v>2.8</v>
+      </c>
+      <c r="G39" s="27">
+        <f t="shared" si="0"/>
+        <v>1.2964088085827217</v>
+      </c>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="36"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>570</v>
+      </c>
+      <c r="B40" s="35">
+        <v>178.9</v>
+      </c>
+      <c r="C40" s="35">
+        <v>180.9</v>
+      </c>
+      <c r="D40" s="35">
+        <v>179.9</v>
+      </c>
+      <c r="E40">
+        <v>2.4</v>
+      </c>
+      <c r="F40">
+        <v>1.6</v>
+      </c>
+      <c r="G40" s="27">
+        <f t="shared" si="0"/>
+        <v>1.276231239577543</v>
+      </c>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="36"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>571</v>
+      </c>
+      <c r="B41" s="35">
+        <v>183.3</v>
+      </c>
+      <c r="C41" s="35">
+        <v>184.6</v>
+      </c>
+      <c r="D41" s="35">
+        <v>184</v>
+      </c>
+      <c r="E41">
+        <v>1.9</v>
+      </c>
+      <c r="F41">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G41" s="27">
+        <f t="shared" si="0"/>
+        <v>1.2477934782608695</v>
+      </c>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
+      <c r="O41" s="36"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>572</v>
+      </c>
+      <c r="B42" s="35">
+        <v>187.6</v>
+      </c>
+      <c r="C42" s="35">
+        <v>190.2</v>
+      </c>
+      <c r="D42" s="35">
+        <v>188.9</v>
+      </c>
+      <c r="E42">
+        <v>3.3</v>
+      </c>
+      <c r="F42">
+        <v>2.7</v>
+      </c>
+      <c r="G42" s="27">
+        <f t="shared" si="0"/>
+        <v>1.2154261514028586</v>
+      </c>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
+      <c r="O42" s="36"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>573</v>
+      </c>
+      <c r="B43" s="35">
+        <v>193.2</v>
+      </c>
+      <c r="C43" s="35">
+        <v>197.4</v>
+      </c>
+      <c r="D43" s="35">
+        <v>195.3</v>
+      </c>
+      <c r="E43">
+        <v>3.4</v>
+      </c>
+      <c r="F43">
+        <v>3.4</v>
+      </c>
+      <c r="G43" s="27">
+        <f t="shared" si="0"/>
+        <v>1.1755965181771633</v>
+      </c>
+      <c r="M43" s="2"/>
+      <c r="N43" s="37"/>
+      <c r="O43" s="36"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>574</v>
+      </c>
+      <c r="B44" s="35">
+        <v>200.6</v>
+      </c>
+      <c r="C44" s="35">
+        <v>202.6</v>
+      </c>
+      <c r="D44" s="35">
+        <v>201.6</v>
+      </c>
+      <c r="E44">
+        <v>2.5</v>
+      </c>
+      <c r="F44">
+        <v>3.2</v>
+      </c>
+      <c r="G44" s="27">
+        <f t="shared" si="0"/>
+        <v>1.1388591269841271</v>
+      </c>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+      <c r="O44" s="36"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>575</v>
+      </c>
+      <c r="B45" s="38">
+        <v>205.709</v>
+      </c>
+      <c r="C45" s="38">
+        <v>208.976</v>
+      </c>
+      <c r="D45" s="38">
+        <v>207.34200000000001</v>
+      </c>
+      <c r="E45">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="F45">
+        <v>2.8</v>
+      </c>
+      <c r="G45" s="27">
+        <f t="shared" si="0"/>
+        <v>1.107320272786025</v>
+      </c>
+      <c r="M45" s="2"/>
+      <c r="N45" s="2"/>
+      <c r="O45" s="36"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>576</v>
+      </c>
+      <c r="B46" s="38">
+        <v>214.429</v>
+      </c>
+      <c r="C46" s="38">
+        <v>216.17699999999999</v>
+      </c>
+      <c r="D46" s="38">
+        <v>215.303</v>
+      </c>
+      <c r="E46">
+        <v>0.1</v>
+      </c>
+      <c r="F46">
+        <v>3.8</v>
+      </c>
+      <c r="G46" s="27">
+        <f t="shared" si="0"/>
+        <v>1.0663762232760343</v>
+      </c>
+      <c r="M46" s="2"/>
+      <c r="N46" s="2"/>
+      <c r="O46" s="36"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>577</v>
+      </c>
+      <c r="B47" s="38">
+        <v>213.13900000000001</v>
+      </c>
+      <c r="C47" s="38">
+        <v>215.935</v>
+      </c>
+      <c r="D47" s="38">
+        <v>214.53700000000001</v>
+      </c>
+      <c r="E47">
+        <v>2.7</v>
+      </c>
+      <c r="F47">
+        <v>-0.4</v>
+      </c>
+      <c r="G47" s="27">
+        <f t="shared" si="0"/>
+        <v>1.0701836979169095</v>
+      </c>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
+      <c r="O47" s="36"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>578</v>
+      </c>
+      <c r="B48" s="38">
+        <v>217.535</v>
+      </c>
+      <c r="C48" s="38">
+        <v>218.57599999999999</v>
+      </c>
+      <c r="D48" s="38">
+        <v>218.05600000000001</v>
+      </c>
+      <c r="E48">
+        <v>1.5</v>
+      </c>
+      <c r="F48">
+        <v>1.6</v>
+      </c>
+      <c r="G48" s="27">
+        <f t="shared" si="0"/>
+        <v>1.0529130131709286</v>
+      </c>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="36"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>579</v>
+      </c>
+      <c r="B49" s="38">
+        <v>223.59800000000001</v>
+      </c>
+      <c r="C49" s="38">
+        <v>226.28</v>
+      </c>
+      <c r="D49" s="38">
+        <v>224.93899999999999</v>
+      </c>
+      <c r="E49">
+        <v>3</v>
+      </c>
+      <c r="F49">
+        <v>3.2</v>
+      </c>
+      <c r="G49" s="27">
+        <f t="shared" si="0"/>
+        <v>1.0206944993976144</v>
+      </c>
+      <c r="M49" s="2"/>
+      <c r="N49" s="2"/>
+      <c r="O49" s="36"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>580</v>
+      </c>
+      <c r="B50" s="38">
+        <v>228.85</v>
+      </c>
+      <c r="C50" s="38">
+        <v>230.33799999999999</v>
+      </c>
+      <c r="D50" s="38">
+        <v>229.59399999999999</v>
+      </c>
+      <c r="E50">
+        <v>1.7</v>
+      </c>
+      <c r="F50">
+        <v>2.1</v>
+      </c>
+      <c r="G50" s="27">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="M50" s="2"/>
+      <c r="N50" s="2"/>
+      <c r="O50" s="36"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>581</v>
+      </c>
+      <c r="B51" s="38">
+        <v>232.36600000000001</v>
+      </c>
+      <c r="C51" s="38">
+        <v>233.548</v>
+      </c>
+      <c r="D51" s="38">
+        <v>232.95699999999999</v>
+      </c>
+      <c r="E51">
+        <v>1.5</v>
+      </c>
+      <c r="F51">
+        <v>1.5</v>
+      </c>
+      <c r="G51" s="27">
+        <f t="shared" si="0"/>
+        <v>0.98556385942470071</v>
+      </c>
+      <c r="M51" s="2"/>
+      <c r="N51" s="2"/>
+      <c r="O51" s="36"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>582</v>
+      </c>
+      <c r="B52" s="38">
+        <v>236.38399999999999</v>
+      </c>
+      <c r="C52" s="38">
+        <v>237.08799999999999</v>
+      </c>
+      <c r="D52" s="38">
+        <v>236.73599999999999</v>
+      </c>
+      <c r="E52">
+        <v>0.8</v>
+      </c>
+      <c r="F52">
+        <v>1.6</v>
+      </c>
+      <c r="G52" s="27">
+        <f t="shared" si="0"/>
+        <v>0.96983137334414704</v>
+      </c>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+      <c r="O52" s="36"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>583</v>
+      </c>
+      <c r="B53" s="38">
+        <v>236.26499999999999</v>
+      </c>
+      <c r="C53" s="38">
+        <v>237.76900000000001</v>
+      </c>
+      <c r="D53" s="38">
+        <v>237.017</v>
+      </c>
+      <c r="E53">
+        <v>0.7</v>
+      </c>
+      <c r="F53">
+        <v>0.1</v>
+      </c>
+      <c r="G53" s="27">
+        <f t="shared" si="0"/>
+        <v>0.9686815713640794</v>
+      </c>
+      <c r="M53" s="2"/>
+      <c r="N53" s="2"/>
+      <c r="O53" s="36"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>584</v>
+      </c>
+      <c r="B54" s="38">
+        <v>238.77799999999999</v>
+      </c>
+      <c r="C54" s="38">
+        <v>241.23699999999999</v>
+      </c>
+      <c r="D54" s="38">
+        <v>240.00700000000001</v>
+      </c>
+      <c r="E54">
+        <v>2.1</v>
+      </c>
+      <c r="F54">
+        <v>1.3</v>
+      </c>
+      <c r="G54" s="27">
+        <f t="shared" si="0"/>
+        <v>0.95661376543184151</v>
+      </c>
+      <c r="M54" s="2"/>
+      <c r="N54" s="2"/>
+      <c r="O54" s="36"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>585</v>
+      </c>
+      <c r="B55" s="38">
+        <v>244.07599999999999</v>
+      </c>
+      <c r="C55" s="38">
+        <v>246.16300000000001</v>
+      </c>
+      <c r="D55" s="38">
+        <v>245.12</v>
+      </c>
+      <c r="E55">
+        <v>2.1</v>
+      </c>
+      <c r="F55">
+        <v>2.1</v>
+      </c>
+      <c r="G55" s="27">
+        <f t="shared" si="0"/>
+        <v>0.93665959530026111</v>
+      </c>
+      <c r="M55" s="2"/>
+      <c r="N55" s="2"/>
+      <c r="O55" s="36"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>586</v>
+      </c>
+      <c r="B56" s="38">
+        <v>250.089</v>
+      </c>
+      <c r="C56" s="38">
+        <v>252.125</v>
+      </c>
+      <c r="D56" s="38">
+        <v>251.107</v>
+      </c>
+      <c r="E56">
+        <v>1.9</v>
+      </c>
+      <c r="F56">
+        <v>2.4</v>
+      </c>
+      <c r="G56" s="27">
+        <f t="shared" si="0"/>
+        <v>0.9143273584567535</v>
+      </c>
+      <c r="M56" s="2"/>
+      <c r="N56" s="2"/>
+      <c r="O56" s="36"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>587</v>
+      </c>
+      <c r="B57" s="38">
+        <v>254.41200000000001</v>
+      </c>
+      <c r="C57" s="38">
+        <v>256.90300000000002</v>
+      </c>
+      <c r="D57" s="38">
+        <v>255.65700000000001</v>
+      </c>
+      <c r="E57">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F57">
+        <v>1.8</v>
+      </c>
+      <c r="G57" s="27">
+        <f t="shared" si="0"/>
+        <v>0.89805481563188172</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>588</v>
+      </c>
+      <c r="B58" s="38">
+        <v>257.55700000000002</v>
+      </c>
+      <c r="C58" s="38">
+        <v>260.065</v>
+      </c>
+      <c r="D58" s="38">
+        <v>258.81099999999998</v>
+      </c>
+      <c r="E58">
+        <v>1.4</v>
+      </c>
+      <c r="F58">
+        <v>1.2</v>
+      </c>
+      <c r="G58" s="27">
+        <f t="shared" si="0"/>
+        <v>0.88711067149387013</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>589</v>
+      </c>
+      <c r="B59" s="38">
+        <v>266.23599999999999</v>
+      </c>
+      <c r="C59" s="38">
+        <v>275.70299999999997</v>
+      </c>
+      <c r="D59" s="38">
+        <v>270.97000000000003</v>
+      </c>
+      <c r="E59">
+        <v>7</v>
+      </c>
+      <c r="F59">
+        <v>4.7</v>
+      </c>
+      <c r="G59" s="27">
+        <f t="shared" si="0"/>
+        <v>0.84730412960844359</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>590</v>
+      </c>
+      <c r="B60" s="38">
+        <v>288.34699999999998</v>
+      </c>
+      <c r="C60" s="38">
+        <v>296.96300000000002</v>
+      </c>
+      <c r="D60" s="38">
+        <v>292.65499999999997</v>
+      </c>
+      <c r="E60">
+        <v>6.5</v>
+      </c>
+      <c r="F60">
+        <v>8</v>
+      </c>
+      <c r="G60" s="27">
+        <f t="shared" si="0"/>
+        <v>0.78452102304761584</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>591</v>
+      </c>
+      <c r="B61" s="38">
+        <v>302.40800000000002</v>
+      </c>
+      <c r="C61" s="38">
+        <v>306.99599999999998</v>
+      </c>
+      <c r="D61" s="38">
+        <v>304.702</v>
+      </c>
+      <c r="G61" s="27">
+        <f t="shared" si="0"/>
+        <v>0.75350342301658668</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>592</v>
+      </c>
+      <c r="B62">
+        <v>312.14499999999998</v>
+      </c>
+      <c r="C62">
+        <v>315.233</v>
+      </c>
+      <c r="D62">
+        <v>313.68900000000002</v>
+      </c>
+      <c r="G62" s="27">
+        <f t="shared" si="0"/>
+        <v>0.73191600598044548</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A366C323-AEA8-47A1-8400-4A398ED6DC8A}">
   <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11828,7 +14786,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79CA3ECE-CC46-4C9C-9910-1D3FD99A313F}">
   <dimension ref="B2:H29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12137,7 +15095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44C2550C-391B-4AED-8625-12FCF8A24E5E}">
   <dimension ref="A1:M90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13696,7 +16654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AB4F1A2-F703-4C6F-AA45-D27647AF57D3}">
   <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14029,7 +16987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2293F3F-9A88-4413-B145-B7568F539BC4}">
   <dimension ref="B2:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14308,7 +17266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5F4C270-6BF9-4D0D-85CD-90AE6754A5FB}">
   <dimension ref="A2:W114"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -16564,7 +19522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1B79DA-1807-4980-8716-C48017AC8EE8}">
   <dimension ref="B2:X23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -17418,914 +20376,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1873BFA-BFB8-479B-8580-77E23D72D642}">
-  <dimension ref="B1:M51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>112</v>
-      </c>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C4" s="12">
-        <v>0.8</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="F4" s="11">
-        <f>D4+$E$6</f>
-        <v>6928</v>
-      </c>
-      <c r="L4" t="s">
-        <v>117</v>
-      </c>
-      <c r="M4" s="1">
-        <f>AVERAGE(H5:H11)</f>
-        <v>7.5361437213570515</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C5" s="12">
-        <v>0.81</v>
-      </c>
-      <c r="D5" s="11">
-        <v>472</v>
-      </c>
-      <c r="F5" s="11">
-        <f t="shared" ref="F5:F11" si="0">D5+$E$6</f>
-        <v>7400</v>
-      </c>
-      <c r="H5">
-        <f>((F5-$F$4)/($F$4))/((C5-$C$4)/($C$4))</f>
-        <v>5.4503464203233207</v>
-      </c>
-      <c r="I5" s="1"/>
-      <c r="L5" t="s">
-        <v>118</v>
-      </c>
-      <c r="M5" s="1">
-        <f>AVERAGE(H13:H17)</f>
-        <v>10.236696165191734</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>117</v>
-      </c>
-      <c r="C6" s="12">
-        <v>0.82</v>
-      </c>
-      <c r="D6">
-        <v>977</v>
-      </c>
-      <c r="E6" s="11">
-        <v>6928</v>
-      </c>
-      <c r="F6" s="11">
-        <f t="shared" si="0"/>
-        <v>7905</v>
-      </c>
-      <c r="H6">
-        <f t="shared" ref="H6:H11" si="1">((F6-$F$4)/($F$4))/((C6-$C$4)/($C$4))</f>
-        <v>5.6408775981524517</v>
-      </c>
-      <c r="I6" s="1"/>
-      <c r="L6" t="s">
-        <v>119</v>
-      </c>
-      <c r="M6" s="1">
-        <f>AVERAGE(H19:H24)</f>
-        <v>7.5709278650378069</v>
-      </c>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C7" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D7" s="11">
-        <v>2759</v>
-      </c>
-      <c r="F7" s="11">
-        <f t="shared" si="0"/>
-        <v>9687</v>
-      </c>
-      <c r="H7">
-        <f t="shared" si="1"/>
-        <v>7.9647806004619088</v>
-      </c>
-      <c r="I7" s="1"/>
-      <c r="L7" t="s">
-        <v>120</v>
-      </c>
-      <c r="M7" s="1">
-        <f>AVERAGE(H26:H29)</f>
-        <v>13.093142804855722</v>
-      </c>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C8" s="12">
-        <v>0.85</v>
-      </c>
-      <c r="D8">
-        <v>3561</v>
-      </c>
-      <c r="F8" s="11">
-        <f t="shared" si="0"/>
-        <v>10489</v>
-      </c>
-      <c r="H8">
-        <f t="shared" si="1"/>
-        <v>8.2240184757505883</v>
-      </c>
-      <c r="I8" s="1"/>
-      <c r="L8" t="s">
-        <v>121</v>
-      </c>
-      <c r="M8" s="1">
-        <f>AVERAGE(H31:H35)</f>
-        <v>6.8445086849877326</v>
-      </c>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C9" s="12">
-        <v>0.93</v>
-      </c>
-      <c r="D9" s="11">
-        <v>10027</v>
-      </c>
-      <c r="F9" s="11">
-        <f t="shared" si="0"/>
-        <v>16955</v>
-      </c>
-      <c r="H9">
-        <f t="shared" si="1"/>
-        <v>8.9065553384260081</v>
-      </c>
-      <c r="I9" s="1"/>
-      <c r="L9" t="s">
-        <v>122</v>
-      </c>
-      <c r="M9" s="1">
-        <f>AVERAGE(H37:H42)</f>
-        <v>4.7753002649653098</v>
-      </c>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C10" s="12">
-        <v>0.95</v>
-      </c>
-      <c r="D10" s="11">
-        <v>10494</v>
-      </c>
-      <c r="F10" s="11">
-        <f t="shared" si="0"/>
-        <v>17422</v>
-      </c>
-      <c r="H10">
-        <f t="shared" si="1"/>
-        <v>8.0785219399538146</v>
-      </c>
-      <c r="I10" s="1"/>
-      <c r="L10" t="s">
-        <v>123</v>
-      </c>
-      <c r="M10" s="1">
-        <f>AVERAGE(H44:H46)</f>
-        <v>10.329147244310422</v>
-      </c>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C11" s="12">
-        <v>0.99</v>
-      </c>
-      <c r="D11" s="11">
-        <v>13966</v>
-      </c>
-      <c r="F11" s="11">
-        <f t="shared" si="0"/>
-        <v>20894</v>
-      </c>
-      <c r="H11">
-        <f t="shared" si="1"/>
-        <v>8.4879056764312661</v>
-      </c>
-      <c r="I11" s="1"/>
-      <c r="L11" t="s">
-        <v>124</v>
-      </c>
-      <c r="M11" s="1">
-        <f>AVERAGE(H48:H50)</f>
-        <v>7.1185033686236947</v>
-      </c>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C12" s="12">
-        <v>0.82</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="F12" s="11">
-        <f>D12+$E$14</f>
-        <v>21244</v>
-      </c>
-    </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C13" s="12">
-        <v>0.83</v>
-      </c>
-      <c r="D13" s="11">
-        <v>2534</v>
-      </c>
-      <c r="F13" s="11">
-        <f t="shared" ref="F13:F17" si="2">D13+$E$14</f>
-        <v>23778</v>
-      </c>
-      <c r="H13">
-        <f>((F13-$F$12)/($F$12))/((C13-$C$12)/($C$12))</f>
-        <v>9.7810205234419048</v>
-      </c>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D14" s="5">
-        <v>5370</v>
-      </c>
-      <c r="E14" s="11">
-        <v>21244</v>
-      </c>
-      <c r="F14" s="11">
-        <f t="shared" si="2"/>
-        <v>26614</v>
-      </c>
-      <c r="H14">
-        <f t="shared" ref="H14:H17" si="3">((F14-$F$12)/($F$12))/((C14-$C$12)/($C$12))</f>
-        <v>10.363867444925617</v>
-      </c>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C15" s="12">
-        <v>0.85</v>
-      </c>
-      <c r="D15" s="11">
-        <v>8544</v>
-      </c>
-      <c r="F15" s="11">
-        <f t="shared" si="2"/>
-        <v>29788</v>
-      </c>
-      <c r="H15">
-        <f t="shared" si="3"/>
-        <v>10.993033327057042</v>
-      </c>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C16" s="12">
-        <v>0.94</v>
-      </c>
-      <c r="D16" s="11">
-        <v>32796</v>
-      </c>
-      <c r="F16" s="11">
-        <f t="shared" si="2"/>
-        <v>54040</v>
-      </c>
-      <c r="H16">
-        <f t="shared" si="3"/>
-        <v>10.549143287516475</v>
-      </c>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C17" s="12">
-        <v>0.97</v>
-      </c>
-      <c r="D17" s="11">
-        <v>36904</v>
-      </c>
-      <c r="F17" s="11">
-        <f t="shared" si="2"/>
-        <v>58148</v>
-      </c>
-      <c r="H17">
-        <f t="shared" si="3"/>
-        <v>9.4964162430176344</v>
-      </c>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="12">
-        <v>0.82</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="F18" s="11">
-        <f>D18+$E$21</f>
-        <v>8404</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C19" s="12">
-        <v>0.83</v>
-      </c>
-      <c r="D19" s="11">
-        <v>634</v>
-      </c>
-      <c r="F19" s="11">
-        <f t="shared" ref="F19:F24" si="4">D19+$E$21</f>
-        <v>9038</v>
-      </c>
-      <c r="H19">
-        <f>((F19-$F$18)/($F$18))/((C19-$C$18)/($C$18))</f>
-        <v>6.1861018562589187</v>
-      </c>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C20" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D20">
-        <v>1315</v>
-      </c>
-      <c r="F20" s="11">
-        <f t="shared" si="4"/>
-        <v>9719</v>
-      </c>
-      <c r="H20">
-        <f t="shared" ref="H20:H24" si="5">((F20-$F$18)/($F$18))/((C20-$C$18)/($C$18))</f>
-        <v>6.4153974297953296</v>
-      </c>
-      <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="12">
-        <v>0.85</v>
-      </c>
-      <c r="D21" s="11">
-        <v>2048</v>
-      </c>
-      <c r="E21" s="11">
-        <v>8404</v>
-      </c>
-      <c r="F21" s="11">
-        <f t="shared" si="4"/>
-        <v>10452</v>
-      </c>
-      <c r="H21">
-        <f t="shared" si="5"/>
-        <v>6.6609551007456709</v>
-      </c>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C22" s="12">
-        <v>0.87</v>
-      </c>
-      <c r="D22">
-        <v>3683</v>
-      </c>
-      <c r="F22" s="11">
-        <f t="shared" si="4"/>
-        <v>12087</v>
-      </c>
-      <c r="H22">
-        <f t="shared" si="5"/>
-        <v>7.1871965730604401</v>
-      </c>
-      <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C23" s="12">
-        <v>0.88</v>
-      </c>
-      <c r="D23" s="11">
-        <v>4594</v>
-      </c>
-      <c r="F23" s="11">
-        <f t="shared" si="4"/>
-        <v>12998</v>
-      </c>
-      <c r="H23">
-        <f t="shared" si="5"/>
-        <v>7.4708075519593775</v>
-      </c>
-      <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C24" s="12">
-        <v>0.97</v>
-      </c>
-      <c r="D24" s="5">
-        <v>17687</v>
-      </c>
-      <c r="F24" s="11">
-        <f t="shared" si="4"/>
-        <v>26091</v>
-      </c>
-      <c r="H24">
-        <f t="shared" si="5"/>
-        <v>11.505108678407106</v>
-      </c>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C25" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="F25" s="11">
-        <f>D25+$E$27</f>
-        <v>18915</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C26" s="12">
-        <v>0.86</v>
-      </c>
-      <c r="D26" s="11">
-        <v>4785</v>
-      </c>
-      <c r="F26" s="11">
-        <f t="shared" ref="F26:F29" si="6">D26+$E$27</f>
-        <v>23700</v>
-      </c>
-      <c r="H26">
-        <f>((F26-$F$25)/($F$25))/((C26-$C$25)/($C$25))</f>
-        <v>10.624900872323542</v>
-      </c>
-      <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>120</v>
-      </c>
-      <c r="C27" s="12">
-        <v>0.88</v>
-      </c>
-      <c r="D27" s="11">
-        <v>10781</v>
-      </c>
-      <c r="E27" s="11">
-        <v>18915</v>
-      </c>
-      <c r="F27" s="11">
-        <f t="shared" si="6"/>
-        <v>29696</v>
-      </c>
-      <c r="H27">
-        <f t="shared" ref="H27:H29" si="7">((F27-$F$25)/($F$25))/((C27-$C$25)/($C$25))</f>
-        <v>11.969389373513073</v>
-      </c>
-      <c r="I27" s="1"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C28" s="12">
-        <v>0.89</v>
-      </c>
-      <c r="D28" s="11">
-        <v>14326</v>
-      </c>
-      <c r="F28" s="11">
-        <f t="shared" si="6"/>
-        <v>33241</v>
-      </c>
-      <c r="H28">
-        <f t="shared" si="7"/>
-        <v>12.724123711340194</v>
-      </c>
-      <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C29" s="12">
-        <v>0.97</v>
-      </c>
-      <c r="D29" s="5">
-        <v>49923</v>
-      </c>
-      <c r="F29" s="11">
-        <f t="shared" si="6"/>
-        <v>68838</v>
-      </c>
-      <c r="H29">
-        <f t="shared" si="7"/>
-        <v>17.054157262246079</v>
-      </c>
-      <c r="I29" s="1"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C30" s="12">
-        <v>0.77</v>
-      </c>
-      <c r="D30">
-        <v>0</v>
-      </c>
-      <c r="F30" s="11">
-        <f>D30+$E$32</f>
-        <v>6659</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C31" s="12">
-        <v>0.78</v>
-      </c>
-      <c r="D31" s="11">
-        <v>540</v>
-      </c>
-      <c r="F31" s="11">
-        <f t="shared" ref="F31:F35" si="8">D31+$E$32</f>
-        <v>7199</v>
-      </c>
-      <c r="H31">
-        <f>((F31-$F$30)/($F$30))/((C31-$C$30)/($C$30))</f>
-        <v>6.244180807929113</v>
-      </c>
-      <c r="I31" s="1"/>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>121</v>
-      </c>
-      <c r="C32" s="12">
-        <v>0.79</v>
-      </c>
-      <c r="D32" s="5">
-        <v>1124</v>
-      </c>
-      <c r="E32" s="11">
-        <v>6659</v>
-      </c>
-      <c r="F32" s="11">
-        <f t="shared" si="8"/>
-        <v>7783</v>
-      </c>
-      <c r="H32">
-        <f t="shared" ref="H32:H35" si="9">((F32-$F$30)/($F$30))/((C32-$C$30)/($C$30))</f>
-        <v>6.4985733593632622</v>
-      </c>
-      <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C33" s="12">
-        <v>0.8</v>
-      </c>
-      <c r="D33" s="11">
-        <v>1756</v>
-      </c>
-      <c r="F33" s="11">
-        <f t="shared" si="8"/>
-        <v>8415</v>
-      </c>
-      <c r="H33">
-        <f t="shared" si="9"/>
-        <v>6.7683836411873592</v>
-      </c>
-      <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C34" s="12">
-        <v>0.81</v>
-      </c>
-      <c r="D34" s="5">
-        <v>2439</v>
-      </c>
-      <c r="F34" s="11">
-        <f t="shared" si="8"/>
-        <v>9098</v>
-      </c>
-      <c r="H34">
-        <f t="shared" si="9"/>
-        <v>7.0507208289532901</v>
-      </c>
-      <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C35" s="12">
-        <v>0.83</v>
-      </c>
-      <c r="D35" s="11">
-        <v>3975</v>
-      </c>
-      <c r="F35" s="11">
-        <f t="shared" si="8"/>
-        <v>10634</v>
-      </c>
-      <c r="H35">
-        <f t="shared" si="9"/>
-        <v>7.6606847875056383</v>
-      </c>
-      <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C36" s="12">
-        <v>0.77</v>
-      </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="F36" s="11">
-        <f>D36+$E$39</f>
-        <v>19122</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C37" s="12">
-        <v>0.78</v>
-      </c>
-      <c r="D37" s="5">
-        <v>1097</v>
-      </c>
-      <c r="F37" s="11">
-        <f t="shared" ref="F37:F42" si="10">D37+$E$39</f>
-        <v>20219</v>
-      </c>
-      <c r="H37">
-        <f>((F37-$F$36)/($F$36))/((C37-$C$36)/($C$36))</f>
-        <v>4.4173726597636191</v>
-      </c>
-      <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C38" s="12">
-        <v>0.79</v>
-      </c>
-      <c r="D38" s="5">
-        <v>2256</v>
-      </c>
-      <c r="F38" s="11">
-        <f t="shared" si="10"/>
-        <v>21378</v>
-      </c>
-      <c r="H38">
-        <f t="shared" ref="H38:H42" si="11">((F38-$F$36)/($F$36))/((C38-$C$36)/($C$36))</f>
-        <v>4.5422026984624999</v>
-      </c>
-      <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>122</v>
-      </c>
-      <c r="C39" s="12">
-        <v>0.8</v>
-      </c>
-      <c r="D39" s="5">
-        <v>3483</v>
-      </c>
-      <c r="E39" s="11">
-        <v>19122</v>
-      </c>
-      <c r="F39" s="11">
-        <f t="shared" si="10"/>
-        <v>22605</v>
-      </c>
-      <c r="H39">
-        <f t="shared" si="11"/>
-        <v>4.67508628804518</v>
-      </c>
-      <c r="I39" s="1"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C40" s="12">
-        <v>0.81</v>
-      </c>
-      <c r="D40">
-        <v>4779</v>
-      </c>
-      <c r="F40" s="11">
-        <f t="shared" si="10"/>
-        <v>23901</v>
-      </c>
-      <c r="H40">
-        <f t="shared" si="11"/>
-        <v>4.8109899592092837</v>
-      </c>
-      <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C41" s="12">
-        <v>0.82</v>
-      </c>
-      <c r="D41" s="11">
-        <v>6150</v>
-      </c>
-      <c r="F41" s="11">
-        <f t="shared" si="10"/>
-        <v>25272</v>
-      </c>
-      <c r="H41">
-        <f t="shared" si="11"/>
-        <v>4.9529337935362481</v>
-      </c>
-      <c r="I41" s="1"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C42" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D42">
-        <v>9132</v>
-      </c>
-      <c r="F42" s="11">
-        <f t="shared" si="10"/>
-        <v>28254</v>
-      </c>
-      <c r="H42">
-        <f t="shared" si="11"/>
-        <v>5.2532161907750279</v>
-      </c>
-      <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C43" s="12">
-        <v>0.81</v>
-      </c>
-      <c r="D43">
-        <v>0</v>
-      </c>
-      <c r="F43" s="11">
-        <f>D43+$E$44</f>
-        <v>7294</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>123</v>
-      </c>
-      <c r="C44" s="12">
-        <v>0.83</v>
-      </c>
-      <c r="D44" s="5">
-        <v>1722</v>
-      </c>
-      <c r="E44" s="11">
-        <v>7294</v>
-      </c>
-      <c r="F44" s="11">
-        <f t="shared" ref="F44:F46" si="12">D44+$E$44</f>
-        <v>9016</v>
-      </c>
-      <c r="H44">
-        <f>((F44-$F$43)/($F$43))/((C44-$C$43)/($C$43))</f>
-        <v>9.5614203454894877</v>
-      </c>
-      <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C45" s="12">
-        <v>0.84</v>
-      </c>
-      <c r="D45">
-        <v>2730</v>
-      </c>
-      <c r="F45" s="11">
-        <f t="shared" si="12"/>
-        <v>10024</v>
-      </c>
-      <c r="H45">
-        <f t="shared" ref="H45:H46" si="13">((F45-$F$43)/($F$43))/((C45-$C$43)/($C$43))</f>
-        <v>10.10556621881001</v>
-      </c>
-      <c r="I45" s="1"/>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C46" s="12">
-        <v>0.86</v>
-      </c>
-      <c r="D46" s="11">
-        <v>5097</v>
-      </c>
-      <c r="F46" s="11">
-        <f t="shared" si="12"/>
-        <v>12391</v>
-      </c>
-      <c r="H46">
-        <f t="shared" si="13"/>
-        <v>11.320455168631767</v>
-      </c>
-      <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C47" s="12">
-        <v>0.81</v>
-      </c>
-      <c r="D47">
-        <v>0</v>
-      </c>
-      <c r="F47" s="11">
-        <f>D47+$E$48</f>
-        <v>18702</v>
-      </c>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>124</v>
-      </c>
-      <c r="C48" s="12">
-        <v>0.83</v>
-      </c>
-      <c r="D48" s="11">
-        <v>3071</v>
-      </c>
-      <c r="E48" s="11">
-        <v>18702</v>
-      </c>
-      <c r="F48" s="11">
-        <f t="shared" ref="F48:F50" si="14">D48+$E$48</f>
-        <v>21773</v>
-      </c>
-      <c r="H48">
-        <f>((F48-$F$47)/($F$47))/((C48-$C$47)/($C$47))</f>
-        <v>6.6503849855630728</v>
-      </c>
-      <c r="I48" s="1"/>
-    </row>
-    <row r="49" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C49" s="12">
-        <v>0.85</v>
-      </c>
-      <c r="D49" s="11">
-        <v>6521</v>
-      </c>
-      <c r="F49" s="11">
-        <f t="shared" si="14"/>
-        <v>25223</v>
-      </c>
-      <c r="H49">
-        <f t="shared" ref="H49:H50" si="15">((F49-$F$47)/($F$47))/((C49-$C$47)/($C$47))</f>
-        <v>7.060755534167483</v>
-      </c>
-      <c r="I49" s="1"/>
-    </row>
-    <row r="50" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C50" s="12">
-        <v>0.87</v>
-      </c>
-      <c r="D50" s="11">
-        <v>10590</v>
-      </c>
-      <c r="F50" s="11">
-        <f t="shared" si="14"/>
-        <v>29292</v>
-      </c>
-      <c r="H50">
-        <f t="shared" si="15"/>
-        <v>7.6443695861405265</v>
-      </c>
-      <c r="I50" s="1"/>
-    </row>
-    <row r="51" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="I51" s="13">
-        <f>AVERAGE(H1:H50)</f>
-        <v>8.126972362529246</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>